<commit_message>
Benchmark de renta fija: Bloomberg U.S. Long Government/Credit Index
Se nombra explícitamente el índice de Bloomberg (el que sigue BLV) como benchmark de la
clase renta fija larga, con 50% TLH + 50% VCLT como proxy invertible, en el análisis,
la sección 3.5 y el Anexo B del informe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5hAYzxrHpdpyuLVyANGG6
</commit_message>
<xml_diff>
--- a/nexum_proyecto_final/resultados/analisis_adicional.xlsx
+++ b/nexum_proyecto_final/resultados/analisis_adicional.xlsx
@@ -580,7 +580,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tesoro y corporativos largos 50/50 (TLH/VCLT)</t>
+          <t>Bloomberg U.S. Long Government/Credit (proxy: 50% TLH + 50% VCLT)</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -748,7 +748,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tesoro y corporativos largos 50/50 (TLH/VCLT)</t>
+          <t>Bloomberg U.S. Long Government/Credit (proxy: 50% TLH + 50% VCLT)</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TLH/VCLT 50/50</t>
+          <t>Bloomberg U.S. Long Gov/Credit (proxy TLH/VCLT 50/50)</t>
         </is>
       </c>
       <c r="I3" t="n">

</xml_diff>

<commit_message>
Benchmark de commodities: DJP (Bloomberg Commodity Index TR)
- config/portafolio/run_all/excel_modelo: el sleeve de commodities se mide contra DJP en
  vez de la mezcla igual ponderada de los 5 ETF; serie DJP agregada a extra_prices.parquet.
- benchmark_djp.py (nuevo): recalcula solo benchmark de política, métricas, tracking error
  y estrategias sobre los retornos oficiales, sin rehacer backtests (estrategias, BL y
  Montecarlo quedan idénticos).
- analisis_adicional e informe: benchmark por clase de commodities = DJP; en vivo sigue la
  mezcla de 5 ETF por falta de precios de DJP posteriores al 11-sep.
- Excel, figuras e informe regenerados; LEEME actualizado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5hAYzxrHpdpyuLVyANGG6
</commit_message>
<xml_diff>
--- a/nexum_proyecto_final/resultados/analisis_adicional.xlsx
+++ b/nexum_proyecto_final/resultados/analisis_adicional.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mezcla igual ponderada GLD/USO/DBA/SLV/CPER</t>
+          <t>Bloomberg Commodity Index TR (DJP)</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -646,37 +646,37 @@
         <v>0.1059737629634363</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1208156329291377</v>
+        <v>0.08518532692572656</v>
       </c>
       <c r="G4" t="n">
         <v>0.1915664201125896</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1527866332264217</v>
+        <v>0.1632473224122437</v>
       </c>
       <c r="I4" t="n">
         <v>0.5122823160508626</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6882536152541703</v>
+        <v>0.4544463080476454</v>
       </c>
       <c r="K4" t="n">
         <v>-0.3143638938037138</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.2979613434248394</v>
+        <v>-0.3617774538943662</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1751620058559213</v>
+        <v>0.1962564546614131</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.04007640397496848</v>
+        <v>0.1220288343904893</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.007019863307747697</v>
+        <v>0.02394894640394216</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.0004289136481033843</v>
+        <v>0.001463280625280866</v>
       </c>
     </row>
     <row r="5">
@@ -804,7 +804,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mezcla igual ponderada GLD/USO/DBA/SLV/CPER</t>
+          <t>Bloomberg Commodity Index TR (DJP)</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -814,37 +814,37 @@
         <v>0.07945914007391841</v>
       </c>
       <c r="F7" t="n">
-        <v>0.04543509449826066</v>
+        <v>0.01597448263457779</v>
       </c>
       <c r="G7" t="n">
         <v>0.1698691890165765</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1535674183827107</v>
+        <v>0.1620741006175871</v>
       </c>
       <c r="I7" t="n">
         <v>0.4395103827339811</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2608214745997808</v>
+        <v>0.07846271010203615</v>
       </c>
       <c r="K7" t="n">
         <v>-0.3143638938037138</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.5443023329311707</v>
+        <v>-0.6163120606390778</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1687044932221787</v>
+        <v>0.1862813204190877</v>
       </c>
       <c r="N7" t="n">
-        <v>0.2051254895787032</v>
+        <v>0.3325212585364167</v>
       </c>
       <c r="O7" t="n">
-        <v>0.03460559176632644</v>
+        <v>0.06194249910758054</v>
       </c>
       <c r="P7" t="n">
-        <v>0.002114401656922546</v>
+        <v>0.003784686695473171</v>
       </c>
     </row>
   </sheetData>
@@ -1304,7 +1304,7 @@
         <v>-0.2047527980997259</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01916660262329831</v>
+        <v>0.01958612254365808</v>
       </c>
       <c r="G2" t="n">
         <v>0.95955</v>
@@ -1332,7 +1332,7 @@
         <v>-0.1842194796204346</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02159554786423215</v>
+        <v>0.02132850227745132</v>
       </c>
       <c r="G3" t="n">
         <v>0.968</v>
@@ -1360,7 +1360,7 @@
         <v>-0.2065461378557338</v>
       </c>
       <c r="F4" t="n">
-        <v>0.01953894764119159</v>
+        <v>0.02014250483446119</v>
       </c>
       <c r="G4" t="n">
         <v>0.9417</v>
@@ -1388,7 +1388,7 @@
         <v>-0.1860669012416921</v>
       </c>
       <c r="F5" t="n">
-        <v>0.02182028225500192</v>
+        <v>0.0217337186288071</v>
       </c>
       <c r="G5" t="n">
         <v>0.9535</v>
@@ -1652,10 +1652,10 @@
         <v>0.6460563579361195</v>
       </c>
       <c r="H2" t="n">
-        <v>0.02893547433451932</v>
+        <v>0.02937528622236973</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.2994792384896898</v>
+        <v>-0.2305808867488592</v>
       </c>
     </row>
     <row r="3">
@@ -1670,19 +1670,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.09461853044171575</v>
+        <v>0.09267204755497915</v>
       </c>
       <c r="D3" t="n">
-        <v>0.109563056609669</v>
+        <v>0.1086374276463029</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6899387144496072</v>
+        <v>0.6783997168545667</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.2139947803662722</v>
+        <v>-0.2032541931862171</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6791364818698666</v>
+        <v>0.6764060351347934</v>
       </c>
       <c r="H3" t="n">
         <v>0.01964224962814203</v>
@@ -1703,19 +1703,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1073361137725004</v>
+        <v>0.1053654065908107</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1161181275582817</v>
+        <v>0.1152757311112064</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7575380141567484</v>
+        <v>0.7466593415198833</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2389402700102807</v>
+        <v>-0.2284993751135759</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7413325795732532</v>
+        <v>0.7386021328381799</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -1749,10 +1749,10 @@
         <v>0.6360681372614863</v>
       </c>
       <c r="H5" t="n">
-        <v>0.02726872327023363</v>
+        <v>0.02770135457134432</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.1288742040113457</v>
+        <v>-0.06656533573321592</v>
       </c>
     </row>
     <row r="6">
@@ -1767,25 +1767,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.0904175086997705</v>
+        <v>0.08868744463033162</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1010364259019764</v>
+        <v>0.100314160324185</v>
       </c>
       <c r="E6" t="n">
-        <v>0.748988491849422</v>
+        <v>0.7377306950530742</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.2139947803662723</v>
+        <v>-0.2032541931862173</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6592853048555198</v>
+        <v>0.6575740958923209</v>
       </c>
       <c r="H6" t="n">
         <v>0.01889319260549622</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.6391951938010439</v>
+        <v>-0.6391951938010437</v>
       </c>
     </row>
     <row r="7">
@@ -1800,19 +1800,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.1028091356329826</v>
+        <v>0.1010570908833262</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1077377060080507</v>
+        <v>0.1070957932623914</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8144925432198319</v>
+        <v>0.8037782858353043</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.2389402700102808</v>
+        <v>-0.2284993751135761</v>
       </c>
       <c r="G7" t="n">
-        <v>0.7277201291642241</v>
+        <v>0.7260089202010254</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Mezcla de 5 ETF</t>
+          <t>Mezcla de 5 ETF (DJP sin precios en vivo)</t>
         </is>
       </c>
       <c r="I4" t="n">

</xml_diff>

<commit_message>
Commodities en vivo contra DJP (precios de Nasdaq.com al 8-oct)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5hAYzxrHpdpyuLVyANGG6
</commit_message>
<xml_diff>
--- a/nexum_proyecto_final/resultados/analisis_adicional.xlsx
+++ b/nexum_proyecto_final/resultados/analisis_adicional.xlsx
@@ -2084,14 +2084,14 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Mezcla de 5 ETF (DJP sin precios en vivo)</t>
+          <t>Bloomberg Commodity Index TR (DJP)</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>-0.01535205629669518</v>
+        <v>-0.01334216502649521</v>
       </c>
       <c r="J4" t="n">
-        <v>-6.582178722759221</v>
+        <v>-6.783167849779219</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Implementación al 14-oct: exports de StockTrak, precios de benchmarks y nuevas desviaciones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5hAYzxrHpdpyuLVyANGG6
</commit_message>
<xml_diff>
--- a/nexum_proyecto_final/resultados/analisis_adicional.xlsx
+++ b/nexum_proyecto_final/resultados/analisis_adicional.xlsx
@@ -20,7 +20,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commodities_califican" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regla_commodities" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activos_adicionales" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control_calendario" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1402,173 +1401,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Versión</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Momentum en acciones CAGR</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Low-Volatility CAGR</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Momentum en commodities CAGR</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Cartera CAGR</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Cartera Sharpe</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>P(3 objetivos) histórico</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>BL SPY</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>BL TLH</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>BL VCLT</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>BL MOM_CMD</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>BL MOM_EQ</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>BL LOW_VOL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Motor oficial (selección de t aplicada de t+1 a t+2)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.1618438769229014</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.1071607336590132</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.07945914007391841</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.09993360885041302</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.8497646103824529</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.95955</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.3726882615883867</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.1708901875389872</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.1484280730577051</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.06594458115755064</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.07023126114771973</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.1718176355096506</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Selección de t aplicada de t a t+1</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.1731429975673637</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.107730783382934</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.05893740312789064</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.09926007028346473</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.8454382730732659</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.9562</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.3721132523534689</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.1689627785682571</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.1467548153807914</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.08074695989087599</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.07432985550184504</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.1570923383047616</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1957,7 +1789,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Valor al 6-oct</t>
+          <t>Valor final</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -1996,19 +1828,19 @@
         <v>86856.63</v>
       </c>
       <c r="C2" t="n">
-        <v>-84203.90730000001</v>
+        <v>-80438.9173</v>
       </c>
       <c r="D2" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E2" t="n">
-        <v>85172.25999999999</v>
+        <v>80967.6597</v>
       </c>
       <c r="F2" t="n">
-        <v>488.3526999999885</v>
+        <v>-11.25759999999718</v>
       </c>
       <c r="G2" t="n">
-        <v>0.00562251494215224</v>
+        <v>-0.0001296112916192717</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -2016,10 +1848,10 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0.0248726509093371</v>
+        <v>0.01163782041389472</v>
       </c>
       <c r="J2" t="n">
-        <v>-1.925013596718486</v>
+        <v>-1.176743170551399</v>
       </c>
     </row>
     <row r="3">
@@ -2038,13 +1870,13 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>43499.68</v>
+        <v>43984.39999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>-1505.337599999999</v>
+        <v>-1020.617600000005</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.03331905546500312</v>
+        <v>-0.02259029099051173</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -2052,10 +1884,10 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>-0.03270257914338592</v>
+        <v>-0.02210561653425236</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.06164763216171959</v>
+        <v>-0.04846744562593749</v>
       </c>
     </row>
     <row r="4">
@@ -2068,19 +1900,19 @@
         <v>8705.76</v>
       </c>
       <c r="C4" t="n">
-        <v>-4669.68</v>
+        <v>-8652.08</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>4003</v>
+        <v>7988.780000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>-706.6800000000003</v>
+        <v>-713.2999999999993</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0811738435242874</v>
+        <v>-0.08193425961662155</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -2088,10 +1920,10 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>-0.01334216502649521</v>
+        <v>-0.005866767600302802</v>
       </c>
       <c r="J4" t="n">
-        <v>-6.783167849779219</v>
+        <v>-7.606749201631875</v>
       </c>
     </row>
     <row r="5">
@@ -2110,13 +1942,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>6931.74</v>
+        <v>6936.915</v>
       </c>
       <c r="F5" t="n">
-        <v>5.90769999999975</v>
+        <v>11.08269999999993</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0008516745307839105</v>
+        <v>0.001597720487214853</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -2124,10 +1956,10 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>0.002300722143403044</v>
+        <v>0.003039355185632031</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.1449047612619134</v>
+        <v>-0.1441634698417178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>